<commit_message>
Passasjertall og puktlighet buss juni 2026
</commit_message>
<xml_diff>
--- a/Data/Mobilitet_i_Telemark/Buss_og_ferge/Punktlighet/RTI_HIST_DETAIL_REGION_LINJE_RAWT_052026.xlsx
+++ b/Data/Mobilitet_i_Telemark/Buss_og_ferge/Punktlighet/RTI_HIST_DETAIL_REGION_LINJE_RAWT_052026.xlsx
@@ -130,13 +130,13 @@
         </is>
       </c>
       <c r="D3" s="1" t="n">
-        <v>944358.0</v>
+        <v>954171.0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>382563.0</v>
+        <v>386674.0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>561795.0</v>
+        <v>567497.0</v>
       </c>
     </row>
     <row r="4">
@@ -270,13 +270,13 @@
         <v>5.0</v>
       </c>
       <c r="D10" s="1" t="n">
-        <v>236665.0</v>
+        <v>240110.0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>107761.0</v>
+        <v>109445.0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>128904.0</v>
+        <v>130665.0</v>
       </c>
     </row>
     <row r="11">
@@ -290,13 +290,13 @@
         <v>5.0</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>101680.0</v>
+        <v>102842.0</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>50540.0</v>
+        <v>51143.0</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>51140.0</v>
+        <v>51699.0</v>
       </c>
     </row>
     <row r="12">
@@ -310,13 +310,13 @@
         <v>5.0</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>117918.0</v>
+        <v>118752.0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>48685.0</v>
+        <v>48859.0</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>69233.0</v>
+        <v>69893.0</v>
       </c>
     </row>
     <row r="13">
@@ -350,13 +350,13 @@
         <v>5.0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>36814.0</v>
+        <v>37174.0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>16821.0</v>
+        <v>17017.0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>19993.0</v>
+        <v>20157.0</v>
       </c>
     </row>
     <row r="15">
@@ -370,13 +370,13 @@
         <v>5.0</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>28932.0</v>
+        <v>29222.0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>7782.0</v>
+        <v>7844.0</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>21150.0</v>
+        <v>21378.0</v>
       </c>
     </row>
     <row r="16">
@@ -390,13 +390,13 @@
         <v>5.0</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>41054.0</v>
+        <v>41540.0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>12687.0</v>
+        <v>12725.0</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>28367.0</v>
+        <v>28815.0</v>
       </c>
     </row>
     <row r="17">
@@ -430,13 +430,13 @@
         <v>5.0</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>14175.0</v>
+        <v>14381.0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>3684.0</v>
+        <v>3740.0</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>10491.0</v>
+        <v>10641.0</v>
       </c>
     </row>
     <row r="19">
@@ -530,13 +530,13 @@
         <v>5.0</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>8220.0</v>
+        <v>8423.0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>4130.0</v>
+        <v>4230.0</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>4090.0</v>
+        <v>4193.0</v>
       </c>
     </row>
     <row r="24">
@@ -910,13 +910,13 @@
         <v>5.0</v>
       </c>
       <c r="D42" s="1" t="n">
-        <v>376.0</v>
+        <v>452.0</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>247.0</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>129.0</v>
+        <v>205.0</v>
       </c>
     </row>
     <row r="43">
@@ -950,13 +950,13 @@
         <v>5.0</v>
       </c>
       <c r="D44" s="1" t="n">
-        <v>1194.0</v>
+        <v>1240.0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>188.0</v>
+        <v>199.0</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>1006.0</v>
+        <v>1041.0</v>
       </c>
     </row>
     <row r="45">
@@ -970,13 +970,13 @@
         <v>5.0</v>
       </c>
       <c r="D45" s="1" t="n">
-        <v>3726.0</v>
+        <v>3921.0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1412.0</v>
+        <v>1474.0</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>2314.0</v>
+        <v>2447.0</v>
       </c>
     </row>
     <row r="46">
@@ -1110,13 +1110,13 @@
         <v>5.0</v>
       </c>
       <c r="D52" s="1" t="n">
-        <v>44176.0</v>
+        <v>44707.0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>19669.0</v>
+        <v>20000.0</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>24507.0</v>
+        <v>24707.0</v>
       </c>
     </row>
     <row r="53">
@@ -1130,13 +1130,13 @@
         <v>5.0</v>
       </c>
       <c r="D53" s="1" t="n">
-        <v>22676.0</v>
+        <v>22999.0</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>12015.0</v>
+        <v>12139.0</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>10661.0</v>
+        <v>10860.0</v>
       </c>
     </row>
     <row r="54">
@@ -1330,13 +1330,13 @@
         <v>5.0</v>
       </c>
       <c r="D63" s="1" t="n">
-        <v>16039.0</v>
+        <v>16301.0</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>3490.0</v>
+        <v>3520.0</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>12549.0</v>
+        <v>12781.0</v>
       </c>
     </row>
     <row r="64">
@@ -1610,13 +1610,13 @@
         <v>5.0</v>
       </c>
       <c r="D77" s="1" t="n">
-        <v>7831.0</v>
+        <v>7952.0</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>4269.0</v>
+        <v>4304.0</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>3562.0</v>
+        <v>3648.0</v>
       </c>
     </row>
     <row r="78">
@@ -1630,13 +1630,13 @@
         <v>5.0</v>
       </c>
       <c r="D78" s="1" t="n">
-        <v>1366.0</v>
+        <v>1435.0</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>466.0</v>
+        <v>502.0</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>900.0</v>
+        <v>933.0</v>
       </c>
     </row>
     <row r="79">
@@ -1730,13 +1730,13 @@
         <v>5.0</v>
       </c>
       <c r="D83" s="1" t="n">
-        <v>14808.0</v>
+        <v>15321.0</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>3232.0</v>
+        <v>3326.0</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>11576.0</v>
+        <v>11995.0</v>
       </c>
     </row>
     <row r="84">
@@ -2372,13 +2372,13 @@
         <v>5.0</v>
       </c>
       <c r="D115" s="1" t="n">
-        <v>2674.0</v>
+        <v>3099.0</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>837.0</v>
+        <v>1126.0</v>
       </c>
       <c r="F115" s="3" t="n">
-        <v>1837.0</v>
+        <v>1973.0</v>
       </c>
     </row>
     <row r="116">
@@ -2392,13 +2392,13 @@
         <v>5.0</v>
       </c>
       <c r="D116" s="1" t="n">
-        <v>1197.0</v>
+        <v>1356.0</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>373.0</v>
+        <v>513.0</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>824.0</v>
+        <v>843.0</v>
       </c>
     </row>
     <row r="117">
@@ -2412,13 +2412,13 @@
         <v>5.0</v>
       </c>
       <c r="D117" s="1" t="n">
-        <v>834.0</v>
+        <v>941.0</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>210.0</v>
+        <v>256.0</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>624.0</v>
+        <v>685.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>